<commit_message>
calendar picker added on cash book entries , remove the bug of keep shhowing suggestions after select the particula account on cash book entries.
</commit_message>
<xml_diff>
--- a/assets/Designs/ledger design.xlsx
+++ b/assets/Designs/ledger design.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ledger-app\ledger\assets\Designs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8AFDC53A-A6FE-4809-82D7-4E554BABF0D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A109EF12-4E0E-43E3-B606-A87CF6349811}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F409F9C7-5A31-4272-A4F0-1B86DC42769C}"/>
   </bookViews>
@@ -389,14 +389,6 @@
     </font>
     <font>
       <b/>
-      <sz val="22"/>
-      <color rgb="FFCC00CC"/>
-      <name val="HGP明朝E"/>
-      <family val="1"/>
-      <charset val="128"/>
-    </font>
-    <font>
-      <b/>
       <sz val="8"/>
       <color rgb="FFCC00CC"/>
       <name val="游ゴシック"/>
@@ -447,6 +439,14 @@
       <family val="3"/>
       <charset val="128"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="22"/>
+      <color rgb="FFFF33CC"/>
+      <name val="HGP明朝E"/>
+      <family val="1"/>
+      <charset val="128"/>
     </font>
   </fonts>
   <fills count="2">
@@ -542,7 +542,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -552,22 +552,19 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
@@ -578,38 +575,32 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -620,9 +611,9 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFFF33CC"/>
+      <color rgb="FF9900CC"/>
       <color rgb="FFCC00CC"/>
-      <color rgb="FF9900CC"/>
-      <color rgb="FFFF33CC"/>
     </mruColors>
   </colors>
   <extLst>
@@ -950,10 +941,10 @@
       </c>
     </row>
     <row r="2" spans="2:9" ht="26.25" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="I2" s="11" t="s">
+      <c r="I2" s="10" t="s">
         <v>49</v>
       </c>
     </row>
@@ -961,7 +952,7 @@
       <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="H3" s="7" t="s">
+      <c r="H3" s="6" t="s">
         <v>4</v>
       </c>
       <c r="I3" t="s">
@@ -969,10 +960,10 @@
       </c>
     </row>
     <row r="4" spans="2:9" x14ac:dyDescent="0.4">
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="H4" s="6" t="s">
         <v>50</v>
       </c>
       <c r="I4" t="s">
@@ -980,30 +971,30 @@
       </c>
     </row>
     <row r="5" spans="2:9" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
     </row>
     <row r="6" spans="2:9" ht="19.5" thickTop="1" x14ac:dyDescent="0.4">
-      <c r="B6" s="14" t="s">
+      <c r="B6" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="15" t="s">
+      <c r="C6" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="D6" s="15"/>
-      <c r="E6" s="15"/>
-      <c r="F6" s="15"/>
-      <c r="G6" s="15"/>
-      <c r="H6" s="14" t="s">
+      <c r="D6" s="18"/>
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="18"/>
+      <c r="H6" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="I6" s="8" t="s">
+      <c r="I6" s="7" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1011,17 +1002,17 @@
       <c r="B7" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="12" t="s">
+      <c r="C7" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="D7" s="12"/>
-      <c r="E7" s="12"/>
-      <c r="F7" s="12"/>
-      <c r="G7" s="12"/>
+      <c r="D7" s="17"/>
+      <c r="E7" s="17"/>
+      <c r="F7" s="17"/>
+      <c r="G7" s="17"/>
       <c r="H7" t="s">
         <v>12</v>
       </c>
-      <c r="I7" s="16" t="s">
+      <c r="I7" s="12" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1029,13 +1020,13 @@
       <c r="B8" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="D8" s="12"/>
-      <c r="E8" s="12"/>
-      <c r="F8" s="12"/>
-      <c r="G8" s="12"/>
+      <c r="C8" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="D8" s="17"/>
+      <c r="E8" s="17"/>
+      <c r="F8" s="17"/>
+      <c r="G8" s="17"/>
       <c r="H8" t="s">
         <v>12</v>
       </c>
@@ -1047,13 +1038,13 @@
       <c r="B9" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="D9" s="12"/>
-      <c r="E9" s="12"/>
-      <c r="F9" s="12"/>
-      <c r="G9" s="12"/>
+      <c r="C9" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="D9" s="17"/>
+      <c r="E9" s="17"/>
+      <c r="F9" s="17"/>
+      <c r="G9" s="17"/>
       <c r="H9" t="s">
         <v>13</v>
       </c>
@@ -1065,13 +1056,13 @@
       <c r="B10" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="D10" s="12"/>
-      <c r="E10" s="12"/>
-      <c r="F10" s="12"/>
-      <c r="G10" s="12"/>
+      <c r="C10" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="D10" s="17"/>
+      <c r="E10" s="17"/>
+      <c r="F10" s="17"/>
+      <c r="G10" s="17"/>
       <c r="H10" t="s">
         <v>15</v>
       </c>
@@ -1083,13 +1074,13 @@
       <c r="B11" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C11" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="D11" s="12"/>
-      <c r="E11" s="12"/>
-      <c r="F11" s="12"/>
-      <c r="G11" s="12"/>
+      <c r="C11" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="D11" s="17"/>
+      <c r="E11" s="17"/>
+      <c r="F11" s="17"/>
+      <c r="G11" s="17"/>
       <c r="H11" t="s">
         <v>17</v>
       </c>
@@ -1101,13 +1092,13 @@
       <c r="B12" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C12" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="D12" s="12"/>
-      <c r="E12" s="12"/>
-      <c r="F12" s="12"/>
-      <c r="G12" s="12"/>
+      <c r="C12" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="D12" s="17"/>
+      <c r="E12" s="17"/>
+      <c r="F12" s="17"/>
+      <c r="G12" s="17"/>
       <c r="H12" t="s">
         <v>19</v>
       </c>
@@ -1119,13 +1110,13 @@
       <c r="B13" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C13" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="D13" s="12"/>
-      <c r="E13" s="12"/>
-      <c r="F13" s="12"/>
-      <c r="G13" s="12"/>
+      <c r="C13" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="D13" s="17"/>
+      <c r="E13" s="17"/>
+      <c r="F13" s="17"/>
+      <c r="G13" s="17"/>
       <c r="H13" t="s">
         <v>21</v>
       </c>
@@ -1137,13 +1128,13 @@
       <c r="B14" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C14" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="D14" s="12"/>
-      <c r="E14" s="12"/>
-      <c r="F14" s="12"/>
-      <c r="G14" s="12"/>
+      <c r="C14" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="D14" s="17"/>
+      <c r="E14" s="17"/>
+      <c r="F14" s="17"/>
+      <c r="G14" s="17"/>
       <c r="H14" t="s">
         <v>23</v>
       </c>
@@ -1155,13 +1146,13 @@
       <c r="B15" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C15" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="D15" s="12"/>
-      <c r="E15" s="12"/>
-      <c r="F15" s="12"/>
-      <c r="G15" s="12"/>
+      <c r="C15" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="D15" s="17"/>
+      <c r="E15" s="17"/>
+      <c r="F15" s="17"/>
+      <c r="G15" s="17"/>
       <c r="H15" t="s">
         <v>25</v>
       </c>
@@ -1173,13 +1164,13 @@
       <c r="B16" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C16" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="D16" s="12"/>
-      <c r="E16" s="12"/>
-      <c r="F16" s="12"/>
-      <c r="G16" s="12"/>
+      <c r="C16" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="D16" s="17"/>
+      <c r="E16" s="17"/>
+      <c r="F16" s="17"/>
+      <c r="G16" s="17"/>
       <c r="H16" t="s">
         <v>27</v>
       </c>
@@ -1191,13 +1182,13 @@
       <c r="B17" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C17" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="D17" s="12"/>
-      <c r="E17" s="12"/>
-      <c r="F17" s="12"/>
-      <c r="G17" s="12"/>
+      <c r="C17" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="D17" s="17"/>
+      <c r="E17" s="17"/>
+      <c r="F17" s="17"/>
+      <c r="G17" s="17"/>
       <c r="H17" t="s">
         <v>29</v>
       </c>
@@ -1209,13 +1200,13 @@
       <c r="B18" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C18" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="D18" s="12"/>
-      <c r="E18" s="12"/>
-      <c r="F18" s="12"/>
-      <c r="G18" s="12"/>
+      <c r="C18" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="D18" s="17"/>
+      <c r="E18" s="17"/>
+      <c r="F18" s="17"/>
+      <c r="G18" s="17"/>
       <c r="H18" t="s">
         <v>31</v>
       </c>
@@ -1227,13 +1218,13 @@
       <c r="B19" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C19" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="D19" s="12"/>
-      <c r="E19" s="12"/>
-      <c r="F19" s="12"/>
-      <c r="G19" s="12"/>
+      <c r="C19" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="D19" s="17"/>
+      <c r="E19" s="17"/>
+      <c r="F19" s="17"/>
+      <c r="G19" s="17"/>
       <c r="H19" t="s">
         <v>33</v>
       </c>
@@ -1245,13 +1236,13 @@
       <c r="B20" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C20" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="D20" s="12"/>
-      <c r="E20" s="12"/>
-      <c r="F20" s="12"/>
-      <c r="G20" s="12"/>
+      <c r="C20" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="D20" s="17"/>
+      <c r="E20" s="17"/>
+      <c r="F20" s="17"/>
+      <c r="G20" s="17"/>
       <c r="H20" t="s">
         <v>35</v>
       </c>
@@ -1263,13 +1254,13 @@
       <c r="B21" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C21" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="D21" s="12"/>
-      <c r="E21" s="12"/>
-      <c r="F21" s="12"/>
-      <c r="G21" s="12"/>
+      <c r="C21" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="D21" s="17"/>
+      <c r="E21" s="17"/>
+      <c r="F21" s="17"/>
+      <c r="G21" s="17"/>
       <c r="H21" t="s">
         <v>37</v>
       </c>
@@ -1281,13 +1272,13 @@
       <c r="B22" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C22" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="D22" s="12"/>
-      <c r="E22" s="12"/>
-      <c r="F22" s="12"/>
-      <c r="G22" s="12"/>
+      <c r="C22" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="D22" s="17"/>
+      <c r="E22" s="17"/>
+      <c r="F22" s="17"/>
+      <c r="G22" s="17"/>
       <c r="H22" t="s">
         <v>39</v>
       </c>
@@ -1296,85 +1287,77 @@
       </c>
     </row>
     <row r="23" spans="2:9" x14ac:dyDescent="0.4">
-      <c r="B23" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="C23" s="21" t="s">
-        <v>45</v>
-      </c>
-      <c r="D23" s="21"/>
-      <c r="E23" s="21"/>
-      <c r="F23" s="21"/>
-      <c r="G23" s="21"/>
-      <c r="H23" s="22" t="s">
+      <c r="B23" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C23" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="D23" s="17"/>
+      <c r="E23" s="17"/>
+      <c r="F23" s="17"/>
+      <c r="G23" s="17"/>
+      <c r="H23" t="s">
         <v>41</v>
       </c>
-      <c r="I23" s="22" t="s">
+      <c r="I23" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="24" spans="2:9" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B24" s="17" t="s">
-        <v>9</v>
-      </c>
-      <c r="C24" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="D24" s="18"/>
-      <c r="E24" s="18"/>
-      <c r="F24" s="18"/>
-      <c r="G24" s="18"/>
-      <c r="H24" s="19" t="s">
+      <c r="B24" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C24" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="D24" s="15"/>
+      <c r="E24" s="15"/>
+      <c r="F24" s="15"/>
+      <c r="G24" s="15"/>
+      <c r="H24" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="I24" s="19" t="s">
+      <c r="I24" s="14" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="25" spans="2:9" x14ac:dyDescent="0.4">
-      <c r="B25" s="9" t="s">
+      <c r="B25" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="H25" s="6">
+      <c r="H25" s="5">
         <f>SUM(H7:H24)</f>
         <v>0</v>
       </c>
-      <c r="I25" s="6">
+      <c r="I25" s="5">
         <v>0</v>
       </c>
     </row>
     <row r="26" spans="2:9" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B26" s="10"/>
-      <c r="C26" s="10"/>
-      <c r="D26" s="10"/>
-      <c r="E26" s="10"/>
-      <c r="F26" s="10"/>
-      <c r="G26" s="10"/>
-      <c r="H26" s="10"/>
-      <c r="I26" s="10"/>
+      <c r="B26" s="9"/>
+      <c r="C26" s="9"/>
+      <c r="D26" s="9"/>
+      <c r="E26" s="9"/>
+      <c r="F26" s="9"/>
+      <c r="G26" s="9"/>
+      <c r="H26" s="9"/>
+      <c r="I26" s="9"/>
     </row>
     <row r="27" spans="2:9" x14ac:dyDescent="0.4">
-      <c r="G27" s="13" t="s">
+      <c r="G27" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="H27" s="13"/>
-      <c r="I27" s="13"/>
+      <c r="H27" s="16"/>
+      <c r="I27" s="16"/>
     </row>
     <row r="28" spans="2:9" x14ac:dyDescent="0.4">
-      <c r="I28" s="6" t="s">
+      <c r="I28" s="5" t="s">
         <v>48</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="C24:G24"/>
-    <mergeCell ref="G27:I27"/>
-    <mergeCell ref="C18:G18"/>
-    <mergeCell ref="C19:G19"/>
-    <mergeCell ref="C20:G20"/>
-    <mergeCell ref="C21:G21"/>
-    <mergeCell ref="C22:G22"/>
-    <mergeCell ref="C23:G23"/>
     <mergeCell ref="C17:G17"/>
     <mergeCell ref="C6:G6"/>
     <mergeCell ref="C7:G7"/>
@@ -1387,6 +1370,14 @@
     <mergeCell ref="C14:G14"/>
     <mergeCell ref="C15:G15"/>
     <mergeCell ref="C16:G16"/>
+    <mergeCell ref="C24:G24"/>
+    <mergeCell ref="G27:I27"/>
+    <mergeCell ref="C18:G18"/>
+    <mergeCell ref="C19:G19"/>
+    <mergeCell ref="C20:G20"/>
+    <mergeCell ref="C21:G21"/>
+    <mergeCell ref="C22:G22"/>
+    <mergeCell ref="C23:G23"/>
   </mergeCells>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>